<commit_message>
Updated README and made minor changes to plotting macros
</commit_message>
<xml_diff>
--- a/Sheets/SimulataneousFitResultsThesis.xlsx
+++ b/Sheets/SimulataneousFitResultsThesis.xlsx
@@ -1,20 +1,21 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10611"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10911"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/samuelgrant/Documents/gm2/EDM/Sheets/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BFE2A1F3-F7BD-D243-B399-37F7F3C128A3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{69095AC6-2D92-9A41-BC8E-41BDB935F306}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="60" yWindow="500" windowWidth="23580" windowHeight="16940" activeTab="1" xr2:uid="{17D71C46-F216-1347-8A90-14C7EE0E0845}"/>
+    <workbookView xWindow="-2900" yWindow="-20060" windowWidth="23580" windowHeight="16940" activeTab="2" xr2:uid="{17D71C46-F216-1347-8A90-14C7EE0E0845}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
     <sheet name="SimultaneousFits" sheetId="2" r:id="rId2"/>
+    <sheet name="Note" sheetId="3" r:id="rId3"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -36,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="152" uniqueCount="26">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="220" uniqueCount="37">
   <si>
     <t>d_EDM</t>
   </si>
@@ -114,6 +115,39 @@
   </si>
   <si>
     <t>d_EDM (S12S18)</t>
+  </si>
+  <si>
+    <t>chi2ndf</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> A_EDM^{BLIND} [mrad]</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> A_{g-2} [mrad]</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> c [mrad]</t>
+  </si>
+  <si>
+    <t>Station</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> value</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> error</t>
+  </si>
+  <si>
+    <t>delta_rest</t>
+  </si>
+  <si>
+    <t>gamma</t>
+  </si>
+  <si>
+    <t>a_mu</t>
+  </si>
+  <si>
+    <t>delta_lab</t>
   </si>
 </sst>
 </file>
@@ -1689,11 +1723,6 @@
     </row>
   </sheetData>
   <mergeCells count="14">
-    <mergeCell ref="F3:G3"/>
-    <mergeCell ref="D4:E4"/>
-    <mergeCell ref="B11:C11"/>
-    <mergeCell ref="D11:E11"/>
-    <mergeCell ref="H37:I37"/>
     <mergeCell ref="B42:C42"/>
     <mergeCell ref="J4:K4"/>
     <mergeCell ref="L4:M4"/>
@@ -1703,6 +1732,11 @@
     <mergeCell ref="C27:D27"/>
     <mergeCell ref="B35:C35"/>
     <mergeCell ref="B4:C4"/>
+    <mergeCell ref="F3:G3"/>
+    <mergeCell ref="D4:E4"/>
+    <mergeCell ref="B11:C11"/>
+    <mergeCell ref="D11:E11"/>
+    <mergeCell ref="H37:I37"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
@@ -2091,4 +2125,541 @@
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C0940890-2326-A847-8B67-0C5BE5C82FC0}">
+  <dimension ref="A1:H32"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
+  <sheetData>
+    <row r="1" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A1" t="s">
+        <v>35</v>
+      </c>
+      <c r="B1" s="2">
+        <v>1.1659208900000001E-3</v>
+      </c>
+    </row>
+    <row r="2" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A2" t="s">
+        <v>34</v>
+      </c>
+      <c r="B2">
+        <f>SQRT(1+(1/B1))</f>
+        <v>29.303431969091314</v>
+      </c>
+    </row>
+    <row r="3" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A3" t="s">
+        <v>33</v>
+      </c>
+      <c r="B3">
+        <f>0.0495092*1000</f>
+        <v>49.5092</v>
+      </c>
+    </row>
+    <row r="4" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A4" t="s">
+        <v>36</v>
+      </c>
+      <c r="B4">
+        <f>B3/B2</f>
+        <v>1.6895358895920907</v>
+      </c>
+    </row>
+    <row r="6" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A6" t="s">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="7" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="B7" t="s">
+        <v>26</v>
+      </c>
+      <c r="C7" t="s">
+        <v>27</v>
+      </c>
+      <c r="E7" t="s">
+        <v>28</v>
+      </c>
+      <c r="G7" t="s">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="8" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A8" t="s">
+        <v>30</v>
+      </c>
+      <c r="B8" t="s">
+        <v>31</v>
+      </c>
+      <c r="C8" t="s">
+        <v>31</v>
+      </c>
+      <c r="D8" t="s">
+        <v>32</v>
+      </c>
+      <c r="E8" t="s">
+        <v>31</v>
+      </c>
+      <c r="F8" t="s">
+        <v>32</v>
+      </c>
+      <c r="G8" t="s">
+        <v>31</v>
+      </c>
+      <c r="H8" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="9" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A9" t="s">
+        <v>11</v>
+      </c>
+      <c r="B9">
+        <v>0.88305</v>
+      </c>
+      <c r="C9">
+        <v>4.3860099999999999E-2</v>
+      </c>
+      <c r="D9">
+        <v>8.7929400000000008E-3</v>
+      </c>
+      <c r="E9">
+        <v>-1.2127800000000001E-3</v>
+      </c>
+      <c r="F9">
+        <v>8.7887799999999995E-3</v>
+      </c>
+      <c r="G9">
+        <v>-1.1474600000000001E-3</v>
+      </c>
+      <c r="H9">
+        <v>6.2268699999999998E-3</v>
+      </c>
+    </row>
+    <row r="10" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A10" t="s">
+        <v>12</v>
+      </c>
+      <c r="B10">
+        <v>0.85123700000000002</v>
+      </c>
+      <c r="C10">
+        <v>1.7480800000000001E-2</v>
+      </c>
+      <c r="D10">
+        <v>9.2295699999999994E-3</v>
+      </c>
+      <c r="E10">
+        <v>5.1927800000000001E-3</v>
+      </c>
+      <c r="F10">
+        <v>9.2193299999999995E-3</v>
+      </c>
+      <c r="G10">
+        <v>-2.07744E-4</v>
+      </c>
+      <c r="H10">
+        <v>6.5330099999999997E-3</v>
+      </c>
+    </row>
+    <row r="11" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A11" t="s">
+        <v>10</v>
+      </c>
+      <c r="B11">
+        <v>0.86763999999999997</v>
+      </c>
+      <c r="C11">
+        <v>3.1270800000000001E-2</v>
+      </c>
+      <c r="D11">
+        <v>6.3663499999999998E-3</v>
+      </c>
+      <c r="E11">
+        <v>1.8536099999999999E-3</v>
+      </c>
+      <c r="F11">
+        <v>6.3613899999999998E-3</v>
+      </c>
+      <c r="G11">
+        <v>-6.9955699999999996E-4</v>
+      </c>
+      <c r="H11">
+        <v>4.5074199999999998E-3</v>
+      </c>
+    </row>
+    <row r="13" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A13" t="s">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="14" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="B14" t="s">
+        <v>26</v>
+      </c>
+      <c r="C14" t="s">
+        <v>27</v>
+      </c>
+      <c r="E14" t="s">
+        <v>28</v>
+      </c>
+      <c r="G14" t="s">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="15" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A15" t="s">
+        <v>30</v>
+      </c>
+      <c r="B15" t="s">
+        <v>31</v>
+      </c>
+      <c r="C15" t="s">
+        <v>31</v>
+      </c>
+      <c r="D15" t="s">
+        <v>32</v>
+      </c>
+      <c r="E15" t="s">
+        <v>31</v>
+      </c>
+      <c r="F15" t="s">
+        <v>32</v>
+      </c>
+      <c r="G15" t="s">
+        <v>31</v>
+      </c>
+      <c r="H15" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="16" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A16" t="s">
+        <v>11</v>
+      </c>
+      <c r="B16">
+        <v>0.57067699999999999</v>
+      </c>
+      <c r="C16">
+        <v>2.5560300000000001E-2</v>
+      </c>
+      <c r="D16">
+        <v>7.5069000000000004E-3</v>
+      </c>
+      <c r="E16">
+        <v>-2.0172499999999999E-3</v>
+      </c>
+      <c r="F16">
+        <v>7.49178E-3</v>
+      </c>
+      <c r="G16">
+        <v>-2.2965899999999998E-3</v>
+      </c>
+      <c r="H16">
+        <v>5.3120900000000002E-3</v>
+      </c>
+    </row>
+    <row r="17" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A17" t="s">
+        <v>12</v>
+      </c>
+      <c r="B17">
+        <v>0.82675100000000001</v>
+      </c>
+      <c r="C17">
+        <v>3.0718100000000002E-2</v>
+      </c>
+      <c r="D17">
+        <v>7.8924200000000007E-3</v>
+      </c>
+      <c r="E17">
+        <v>-1.01289E-2</v>
+      </c>
+      <c r="F17">
+        <v>7.88698E-3</v>
+      </c>
+      <c r="G17">
+        <v>-1.81909E-3</v>
+      </c>
+      <c r="H17">
+        <v>5.5873600000000004E-3</v>
+      </c>
+    </row>
+    <row r="18" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A18" t="s">
+        <v>10</v>
+      </c>
+      <c r="B18">
+        <v>0.69826999999999995</v>
+      </c>
+      <c r="C18">
+        <v>2.80253E-2</v>
+      </c>
+      <c r="D18">
+        <v>5.4394300000000003E-3</v>
+      </c>
+      <c r="E18">
+        <v>-5.8769399999999998E-3</v>
+      </c>
+      <c r="F18">
+        <v>5.4318600000000002E-3</v>
+      </c>
+      <c r="G18">
+        <v>-2.06347E-3</v>
+      </c>
+      <c r="H18">
+        <v>3.84987E-3</v>
+      </c>
+    </row>
+    <row r="20" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A20" t="s">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="21" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="B21" t="s">
+        <v>26</v>
+      </c>
+      <c r="C21" t="s">
+        <v>27</v>
+      </c>
+      <c r="E21" t="s">
+        <v>28</v>
+      </c>
+      <c r="G21" t="s">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="22" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A22" t="s">
+        <v>30</v>
+      </c>
+      <c r="B22" t="s">
+        <v>31</v>
+      </c>
+      <c r="C22" t="s">
+        <v>31</v>
+      </c>
+      <c r="D22" t="s">
+        <v>32</v>
+      </c>
+      <c r="E22" t="s">
+        <v>31</v>
+      </c>
+      <c r="F22" t="s">
+        <v>32</v>
+      </c>
+      <c r="G22" t="s">
+        <v>31</v>
+      </c>
+      <c r="H22" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="23" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A23" t="s">
+        <v>11</v>
+      </c>
+      <c r="B23">
+        <v>1.0548599999999999</v>
+      </c>
+      <c r="C23">
+        <v>4.8196799999999998E-2</v>
+      </c>
+      <c r="D23">
+        <v>6.1602799999999997E-3</v>
+      </c>
+      <c r="E23">
+        <v>4.0131699999999999E-4</v>
+      </c>
+      <c r="F23">
+        <v>6.1536000000000004E-3</v>
+      </c>
+      <c r="G23">
+        <v>3.6478299999999999E-3</v>
+      </c>
+      <c r="H23">
+        <v>4.3609800000000004E-3</v>
+      </c>
+    </row>
+    <row r="24" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A24" t="s">
+        <v>12</v>
+      </c>
+      <c r="B24">
+        <v>1.4328399999999999</v>
+      </c>
+      <c r="C24">
+        <v>4.3546599999999998E-2</v>
+      </c>
+      <c r="D24">
+        <v>6.53238E-3</v>
+      </c>
+      <c r="E24">
+        <v>-2.7177899999999999E-3</v>
+      </c>
+      <c r="F24">
+        <v>6.5260400000000003E-3</v>
+      </c>
+      <c r="G24">
+        <v>4.2183400000000001E-3</v>
+      </c>
+      <c r="H24">
+        <v>4.62364E-3</v>
+      </c>
+    </row>
+    <row r="25" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A25" t="s">
+        <v>10</v>
+      </c>
+      <c r="B25">
+        <v>1.4193199999999999</v>
+      </c>
+      <c r="C25">
+        <v>4.5993899999999997E-2</v>
+      </c>
+      <c r="D25">
+        <v>4.48183E-3</v>
+      </c>
+      <c r="E25">
+        <v>-1.07424E-3</v>
+      </c>
+      <c r="F25">
+        <v>4.47716E-3</v>
+      </c>
+      <c r="G25">
+        <v>3.9147299999999999E-3</v>
+      </c>
+      <c r="H25">
+        <v>3.1725099999999999E-3</v>
+      </c>
+    </row>
+    <row r="27" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A27" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="28" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="B28" t="s">
+        <v>26</v>
+      </c>
+      <c r="C28" t="s">
+        <v>27</v>
+      </c>
+      <c r="E28" t="s">
+        <v>28</v>
+      </c>
+      <c r="G28" t="s">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="29" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A29" t="s">
+        <v>30</v>
+      </c>
+      <c r="B29" t="s">
+        <v>31</v>
+      </c>
+      <c r="C29" t="s">
+        <v>31</v>
+      </c>
+      <c r="D29" t="s">
+        <v>32</v>
+      </c>
+      <c r="E29" t="s">
+        <v>31</v>
+      </c>
+      <c r="F29" t="s">
+        <v>32</v>
+      </c>
+      <c r="G29" t="s">
+        <v>31</v>
+      </c>
+      <c r="H29" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="30" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A30" t="s">
+        <v>11</v>
+      </c>
+      <c r="B30">
+        <v>0.77335799999999999</v>
+      </c>
+      <c r="C30">
+        <v>3.4760399999999997E-2</v>
+      </c>
+      <c r="D30">
+        <v>5.4018099999999999E-3</v>
+      </c>
+      <c r="E30">
+        <v>7.9582899999999998E-3</v>
+      </c>
+      <c r="F30">
+        <v>5.3944500000000003E-3</v>
+      </c>
+      <c r="G30">
+        <v>1.65763E-3</v>
+      </c>
+      <c r="H30">
+        <v>3.8233299999999998E-3</v>
+      </c>
+    </row>
+    <row r="31" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A31" t="s">
+        <v>12</v>
+      </c>
+      <c r="B31">
+        <v>0.46556700000000001</v>
+      </c>
+      <c r="C31">
+        <v>3.0622099999999999E-2</v>
+      </c>
+      <c r="D31">
+        <v>5.7343400000000001E-3</v>
+      </c>
+      <c r="E31" s="2">
+        <v>-7.1671299999999999E-6</v>
+      </c>
+      <c r="F31">
+        <v>5.7283000000000004E-3</v>
+      </c>
+      <c r="G31">
+        <v>-1.49455E-4</v>
+      </c>
+      <c r="H31">
+        <v>4.0587699999999997E-3</v>
+      </c>
+    </row>
+    <row r="32" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A32" t="s">
+        <v>10</v>
+      </c>
+      <c r="B32">
+        <v>0.62349500000000002</v>
+      </c>
+      <c r="C32">
+        <v>3.2809499999999998E-2</v>
+      </c>
+      <c r="D32">
+        <v>3.9319899999999998E-3</v>
+      </c>
+      <c r="E32">
+        <v>4.2053200000000002E-3</v>
+      </c>
+      <c r="F32">
+        <v>3.9272200000000004E-3</v>
+      </c>
+      <c r="G32">
+        <v>8.0419499999999995E-4</v>
+      </c>
+      <c r="H32">
+        <v>2.7830400000000001E-3</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
 </file>
</xml_diff>